<commit_message>
refactor save monthly sheet statistic
</commit_message>
<xml_diff>
--- a/smart-admin-api-java17-springboot3/月度报表.xlsx
+++ b/smart-admin-api-java17-springboot3/月度报表.xlsx
@@ -8,6 +8,8 @@
   <sheets>
     <sheet name="每月统计" r:id="rId3" sheetId="1"/>
     <sheet name="每月机台服务返仓喷头统计" r:id="rId4" sheetId="2"/>
+    <sheet name="当月破损仓喷头信息" r:id="rId5" sheetId="3"/>
+    <sheet name="每月各机台喷头维护明细" r:id="rId6" sheetId="4"/>
   </sheets>
 </workbook>
 </file>
@@ -18,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-MM-dd"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -31,6 +35,10 @@
       <name val="宋体"/>
       <sz val="14.0"/>
       <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
     </font>
   </fonts>
   <fills count="4">
@@ -79,12 +87,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true">
       <alignment horizontal="center" wrapText="true" vertical="center"/>
       <protection locked="true"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -592,7 +601,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>65.0</v>
+        <v>8.0</v>
       </c>
       <c r="C16" t="n">
         <v>118.0</v>
@@ -3026,4 +3035,2328 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E54"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>年份月份</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>喷头序列号</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>破损机台</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>破损原因</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>破损日期</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>316814-05</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>RMA-沙印2#大机 O17   张仕智</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>活性堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>45699.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>286619-12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RMA-稽山1#大机 LK38   李刚</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>内色差或持续性差</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>45699.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>287133-14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RMA-华都2#大机 O4   陆铭辉</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>45699.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>300451-10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>RMA-绍肖2#大机 O28   胡斌</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>45699.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>271324-05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>RMA-鸿大北海3#大机 B36   谭冬</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>45699.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>298771-17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>RMA-大昌祥2#大机 K36   谭冬</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>活性堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>45699.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>319250-10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RMA-鸿大北海2#大机 C36   卢伟</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>45699.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>287061-07</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>宇华1#大机 O36   马进</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>305227-08</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 K35   卢伟</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>278330-06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 O1   卢伟</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>内色差或持续性差</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>286140-10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 O33   卢伟</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>287685-20</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 B32   卢伟</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>290339-11</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 LK2   卢伟</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>287809-16</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 LK4   卢伟</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>290028-13</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 LK32   卢伟</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>286935-04</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>鸿大北海1#大机 O1   卢伟</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>273931-09</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>鸿大北海2#大机 Y35   卢伟</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>289883-08</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>鸿大北海2#大机 O36   卢伟</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>272467-03</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>鸿大北海2#大机 B37   卢伟</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>289063-09</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>鸿大北海2#大机 LK1   卢伟</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>45700.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>295254-15</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>吉盛祥1#大机 K35   管石岩</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>45701.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>271324-04</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>宇华3#大机 LK36   马进</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>45703.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>292374-04</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>鸿大北海1#小机 K2   卢伟</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>45703.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>225985-10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>宇华2#大机 O36   马进</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>报错驱动过流</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>45705.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>270980-07</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>宇华1#大机 O38   马进</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>45705.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>287029-12</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>鸿大北海1#小机 K2   卢伟</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>45705.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>279572-09</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>鸿大北海1#小机 C1   卢伟</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>45705.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>286680-17</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>宇华1#大机 O40   余正红</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>报错驱动过流</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>45705.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>223719-01</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>大昌德2#大机 Y36   曹骏杰</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>45705.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>303760-15</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>绍肖2#大机 M1   胡斌</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>45707.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>280948-05</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>鸿大北海3#大机 C36   卢伟</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>45707.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>279580-02</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>鸿大北海3#大机 C4   卢伟</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>活性堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>45707.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>306048-19</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>鸿大北海3#大机 C7   谭冬</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>45707.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>292374-12</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>绍肖1#大机 C36 李刚</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>45707.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>297216-01</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>宇华1#大机 LK37   马进</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>45707.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>286721-15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>宇华1#大机 O37   马进</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>报错驱动过流</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>45708.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>295439-01</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>吉盛祥2#大机 Y35   陆铭辉</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>45708.0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>304523-18</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>宏强1#大机 B20   韩志涛</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>内色差或持续性差</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>45708.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>273749-05</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>宏强1#大机 B20   韩志涛</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>45708.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>313941-14</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>鸿大北海2#大机 LK16   卢伟</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>活性湿浆堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>45709.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>289947-20</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>吉盛祥1#大机 LK1   马进</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>45709.0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>316431-20</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>鸿大北海1#小机 O1   卢伟</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>45712.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>288547-21</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>RMA-宇华2#大机 M35   马进</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>内色差或持续性差</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>45712.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>291947-15</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>RMA-大昌祥2#大机 K15   谭冬</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>活性堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>45712.0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>293052-01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>RMA-大昌祥2#大机 B17   谭冬</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>活性堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>45712.0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>292370-12</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>RMA-绍肖1#大机 O5   胡斌</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>活性堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>45712.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>288033-20</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>宇华2#大机 M17   张文江</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>金手指损坏</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>45713.0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>288046-16</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>绍肖2#大机 B36   高至桥</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>活性堵嘴歪针</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>45713.0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>314128-06</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>鸿大北海1#小机 C1   卢伟</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>45713.0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>293150-20</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>大昌祥2#大机 O10   谭冬</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>45714.0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>292374-05</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>大昌祥2#大机 O15   谭冬</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>电路受损</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>45714.0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>290959-08</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>大昌祥扫描机 Y1   谭冬</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>45715.0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>313943-17</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>鸿大北海2#大机 LK8   卢伟</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>物理破损</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>45715.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:AT6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>年份月份</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>维护结果分类</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>大昌德1#</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>大昌德2#</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>宇华1#</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>宇华2#</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>宇华3#</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>华都1#</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>华都2#</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大大昌祥1#</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大大昌祥2#</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大大昌祥扫描机</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大北海1#</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大北海2#</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大北海3#</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>吉盛祥1#</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>吉盛祥2#</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>绍肖1#</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>绍肖2#</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>绍肖3#</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>绍肖4#</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>沙印1#</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>沙印2#</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>宏强1#</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>宏强2#</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>宏强3#</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>稽山1#</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>稽山2#</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>盛兴1#</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>盛兴2#</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>超超1#</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>超超2#</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>宜滨1#</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>宜滨2#</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>恒晨1#</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>恒晨3C1#</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>洁彩坊一号车间1#大机</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>洁彩坊二号车间1#大机</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>金楚1#大机</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大北海1#小机</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大北海2#小机</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大北海3#小机</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>鸿大北海5#小机</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>轮转机</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>共计</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>清洗好可用</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>26.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>破损</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>52.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RMA</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>维护中</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>43.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>小计</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>126.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>